<commit_message>
feat: atualizando estrutura do relatório e respectiva especificação
</commit_message>
<xml_diff>
--- a/report/Relatório_Operacional.xlsx
+++ b/report/Relatório_Operacional.xlsx
@@ -1,22 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4fee7ff2b33926f3/Documentos/Aprendizado/Data/data-platform-gen-1/report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="43" documentId="11_AD4D361C20488DEA4E38A07F349E7EBC5BDEDD8D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC903991-1409-453A-9D04-84068DADE9A4}"/>
+  <xr:revisionPtr revIDLastSave="47" documentId="11_AD4D361C20488DEA4E38A07F349E7EBC5BDEDD8D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2BCD4DC3-665D-498A-8EAD-05CF447367B2}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="VENDAS" sheetId="8" r:id="rId1"/>
-    <sheet name="PRODUTOS" sheetId="2" r:id="rId2"/>
-    <sheet name="CLIENTES" sheetId="3" r:id="rId3"/>
-    <sheet name="VENDEDORES" sheetId="4" r:id="rId4"/>
+    <sheet name="DASHBOARD" sheetId="8" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -75,6 +72,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -345,31 +346,4 @@
   <sheetData/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E8D8D30-E901-438B-A6F9-F5DC0365C943}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A7F740E-287F-4BE0-8C41-6BE2B3194805}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79122337-96E8-4487-A0C3-96F87398DAF1}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
 </file>
</xml_diff>